<commit_message>
Update NY gaming data - Fri Oct 23 15:20:58 UTC 2026
</commit_message>
<xml_diff>
--- a/NY_State_Reports_2026-10-23/DraftKings_Sport_Book_Weekly_Report.xlsx
+++ b/NY_State_Reports_2026-10-23/DraftKings_Sport_Book_Weekly_Report.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="R:\MOBILE SPORTS WAGERING\11_Weekly Web Reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99A0C708-EE64-433B-8D16-F43D1E7D8A62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B71236B-8D77-4EDE-813E-9D60CBB04388}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{EDA5EF8F-B63B-4D9E-966F-AB4A019BBE74}"/>
   </bookViews>
@@ -2815,7 +2815,12 @@
         <v>46313</v>
       </c>
       <c r="B42" s="20"/>
-      <c r="F42" s="33"/>
+      <c r="C42" s="21">
+        <v>208456404.81</v>
+      </c>
+      <c r="F42" s="33">
+        <v>20863203.190000009</v>
+      </c>
       <c r="G42"/>
       <c r="H42"/>
       <c r="I42"/>
@@ -3335,11 +3340,11 @@
       </c>
       <c r="C67" s="23">
         <f>SUM(C13:C66)</f>
-        <v>4887710044.7700005</v>
+        <v>5096166449.5800009</v>
       </c>
       <c r="F67" s="23">
         <f>SUM(F13:F66)</f>
-        <v>421123734.44859982</v>
+        <v>441986937.63859981</v>
       </c>
       <c r="G67"/>
       <c r="H67"/>

</xml_diff>